<commit_message>
Outcomes spreadsheet: list completed trades only
Skipped trades and trades without a result yet are no longer listed on the
Live Mock Trades sheet, and the 'Not resolved / skipped' totals column is
removed. A trade appears once its result is known. Phil's request, 27 Oct 2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013c3SgyzuGU5kun14SDE44S
</commit_message>
<xml_diff>
--- a/docs/examples/ftse_outcomes_synthetic.xlsx
+++ b/docs/examples/ftse_outcomes_synthetic.xlsx
@@ -81,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -100,7 +100,6 @@
     <xf numFmtId="164" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -615,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -648,14 +647,14 @@
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated SYNTHETIC FIXTURE: no observed market performance. The live mock trader enters ideas as they trigger during the day: one new trade per scan, up to 5 a day (3 a day before 23 Oct 2026), one per share, FTSE 100 shares only from 23 Oct 2026, and only ideas that pass the entry rules, including the check that the target would pay more than the stop could cost after costs. Each entry was saved the moment the scan ran (scan_data/live_mock_trades.csv) and is filled at the open of the next 15-minute candle. Trades close at the target, the stop, or the end of the day.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1">
+          <t>Generated SYNTHETIC FIXTURE: no observed market performance. The live mock trader enters ideas as they trigger during the day: every idea that passes the rules, up to 5 open at once and 10 a day (before 26 Oct 2026: 1 new trade per scan and 5 a day; before 23 Oct: 3 a day), one per share, FTSE 100 shares only from 23 Oct 2026, and only ideas that pass the entry rules, including the check that the target would pay more than the stop could cost after costs. Each entry was saved the moment the scan ran (scan_data/live_mock_trades.csv) and is filled at the open of the next 15-minute candle. Trades close at the target, the stop, or the end of the day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Each trade is £100. Dealing costs = 0.10% (buy and sell together); stamp duty = 0.50% on buys of real shares (sells never pay it). Grey rows were never entered or have no result yet.</t>
+          <t>Each trade is £100. Dealing costs = 0.10% (buy and sell together); stamp duty = 0.50% on buys (0 = spread bet, the basis for all results from 26 Oct 2026, including earlier trades). Only completed trades are listed: skipped trades and those without a result yet are left out. Results rechecked with version 3 missing-price safeguards; older totals may differ. Only resolved trades enter the totals.</t>
         </is>
       </c>
     </row>
@@ -687,20 +686,15 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Not resolved / skipped</t>
+          <t>Gross profit / loss (£)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Gross profit / loss (£)</t>
+          <t>Dealing costs (£)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Dealing costs (£)</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Stamp duty (£)</t>
         </is>
@@ -722,16 +716,13 @@
       <c r="E5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="1" t="n">
-        <v>3</v>
+      <c r="F5" s="4" t="n">
+        <v>2.7</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>2.7</v>
+        <v>-0.4</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="I5" s="4" t="n">
         <v>-1.5</v>
       </c>
     </row>
@@ -1174,151 +1165,6 @@
       </c>
       <c r="R16" s="11" t="n">
         <v>0.8</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>10:31</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>Synthetic example 6</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>DEMO5.L</t>
-        </is>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>Long</t>
-        </is>
-      </c>
-      <c r="G17" s="12" t="inlineStr">
-        <is>
-          <t>Range</t>
-        </is>
-      </c>
-      <c r="H17" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="I17" s="12" t="n">
-        <v>98</v>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>106</v>
-      </c>
-      <c r="K17" s="12" t="inlineStr">
-        <is>
-          <t>No data</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>10:31</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>Synthetic example 7</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>DEMO6.L</t>
-        </is>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>Long</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="inlineStr">
-        <is>
-          <t>Breakout</t>
-        </is>
-      </c>
-      <c r="H18" s="12" t="n"/>
-      <c r="I18" s="12" t="n">
-        <v>98</v>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>106</v>
-      </c>
-      <c r="K18" s="12" t="inlineStr">
-        <is>
-          <t>Not resolved yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>10:31</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>Synthetic example 5</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>DEMO4.L</t>
-        </is>
-      </c>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>Long</t>
-        </is>
-      </c>
-      <c r="G19" s="12" t="inlineStr">
-        <is>
-          <t>Breakout</t>
-        </is>
-      </c>
-      <c r="H19" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="I19" s="12" t="n">
-        <v>98</v>
-      </c>
-      <c r="J19" s="12" t="n">
-        <v>106</v>
-      </c>
-      <c r="K19" s="12" t="inlineStr">
-        <is>
-          <t>Skipped (price already past stop or target)</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -1352,7 +1198,7 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Live: trades at trigger points (up to 5 a day) (cumulative £)</t>
+          <t>Live: trades at trigger points (cumulative £)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Outcomes spreadsheet: list completed trades only (#66)
Skipped trades and trades without a result yet are no longer listed on the
Live Mock Trades sheet, and the 'Not resolved / skipped' totals column is
removed. A trade appears once its result is known. Phil's request, 27 Oct 2026.


Claude-Session: https://claude.ai/code/session_013c3SgyzuGU5kun14SDE44S

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/examples/ftse_outcomes_synthetic.xlsx
+++ b/docs/examples/ftse_outcomes_synthetic.xlsx
@@ -81,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -100,7 +100,6 @@
     <xf numFmtId="164" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -615,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -648,14 +647,14 @@
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated SYNTHETIC FIXTURE: no observed market performance. The live mock trader enters ideas as they trigger during the day: one new trade per scan, up to 5 a day (3 a day before 23 Oct 2026), one per share, FTSE 100 shares only from 23 Oct 2026, and only ideas that pass the entry rules, including the check that the target would pay more than the stop could cost after costs. Each entry was saved the moment the scan ran (scan_data/live_mock_trades.csv) and is filled at the open of the next 15-minute candle. Trades close at the target, the stop, or the end of the day.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1">
+          <t>Generated SYNTHETIC FIXTURE: no observed market performance. The live mock trader enters ideas as they trigger during the day: every idea that passes the rules, up to 5 open at once and 10 a day (before 26 Oct 2026: 1 new trade per scan and 5 a day; before 23 Oct: 3 a day), one per share, FTSE 100 shares only from 23 Oct 2026, and only ideas that pass the entry rules, including the check that the target would pay more than the stop could cost after costs. Each entry was saved the moment the scan ran (scan_data/live_mock_trades.csv) and is filled at the open of the next 15-minute candle. Trades close at the target, the stop, or the end of the day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Each trade is £100. Dealing costs = 0.10% (buy and sell together); stamp duty = 0.50% on buys of real shares (sells never pay it). Grey rows were never entered or have no result yet.</t>
+          <t>Each trade is £100. Dealing costs = 0.10% (buy and sell together); stamp duty = 0.50% on buys (0 = spread bet, the basis for all results from 26 Oct 2026, including earlier trades). Only completed trades are listed: skipped trades and those without a result yet are left out. Results rechecked with version 3 missing-price safeguards; older totals may differ. Only resolved trades enter the totals.</t>
         </is>
       </c>
     </row>
@@ -687,20 +686,15 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Not resolved / skipped</t>
+          <t>Gross profit / loss (£)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Gross profit / loss (£)</t>
+          <t>Dealing costs (£)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Dealing costs (£)</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Stamp duty (£)</t>
         </is>
@@ -722,16 +716,13 @@
       <c r="E5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="1" t="n">
-        <v>3</v>
+      <c r="F5" s="4" t="n">
+        <v>2.7</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>2.7</v>
+        <v>-0.4</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="I5" s="4" t="n">
         <v>-1.5</v>
       </c>
     </row>
@@ -1174,151 +1165,6 @@
       </c>
       <c r="R16" s="11" t="n">
         <v>0.8</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>10:31</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>Synthetic example 6</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>DEMO5.L</t>
-        </is>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>Long</t>
-        </is>
-      </c>
-      <c r="G17" s="12" t="inlineStr">
-        <is>
-          <t>Range</t>
-        </is>
-      </c>
-      <c r="H17" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="I17" s="12" t="n">
-        <v>98</v>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>106</v>
-      </c>
-      <c r="K17" s="12" t="inlineStr">
-        <is>
-          <t>No data</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>10:31</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>Synthetic example 7</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>DEMO6.L</t>
-        </is>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>Long</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="inlineStr">
-        <is>
-          <t>Breakout</t>
-        </is>
-      </c>
-      <c r="H18" s="12" t="n"/>
-      <c r="I18" s="12" t="n">
-        <v>98</v>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>106</v>
-      </c>
-      <c r="K18" s="12" t="inlineStr">
-        <is>
-          <t>Not resolved yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>10:31</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>Synthetic example 5</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>DEMO4.L</t>
-        </is>
-      </c>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>Long</t>
-        </is>
-      </c>
-      <c r="G19" s="12" t="inlineStr">
-        <is>
-          <t>Breakout</t>
-        </is>
-      </c>
-      <c r="H19" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="I19" s="12" t="n">
-        <v>98</v>
-      </c>
-      <c r="J19" s="12" t="n">
-        <v>106</v>
-      </c>
-      <c r="K19" s="12" t="inlineStr">
-        <is>
-          <t>Skipped (price already past stop or target)</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -1352,7 +1198,7 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Live: trades at trigger points (up to 5 a day) (cumulative £)</t>
+          <t>Live: trades at trigger points (cumulative £)</t>
         </is>
       </c>
     </row>

</xml_diff>